<commit_message>
Lead extraction 2026-08-06 (weekly, slk)
</commit_message>
<xml_diff>
--- a/UT/slk/2026-08-06.xlsx
+++ b/UT/slk/2026-08-06.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,11 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>Posted Date</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>Property Value</t>
         </is>
       </c>
@@ -512,6 +517,11 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>$ 1,573,400</t>
         </is>
       </c>
@@ -559,6 +569,11 @@
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>$ 475,900</t>
         </is>

</xml_diff>